<commit_message>
remove CNS_ON_STUDY_INITIAL_DIAGNOSIS.SUPPTU_QVAL_TUPTDZSTG from tumor_spatial_extent
</commit_message>
<xml_diff>
--- a/docs/mci_cog_igm_rules_dcc.xlsx
+++ b/docs/mci_cog_igm_rules_dcc.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bullenca/Work/Repos/ChildhoodCancerDataInitiative-Prefect_Pipeline/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BC71A2C-0CF6-BC43-8A8F-365880FB89B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD70575D-8A14-EA40-9085-C81D54A2B95D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4080" yWindow="1420" windowWidth="30240" windowHeight="18980" xr2:uid="{9DC53540-95BC-6744-B593-4545FF261AF8}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2055" uniqueCount="222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2055" uniqueCount="221">
   <si>
     <t>source</t>
   </si>
@@ -280,9 +280,6 @@
   </si>
   <si>
     <t>sts_dx</t>
-  </si>
-  <si>
-    <t>COG_UPR_DX.REG_STAGE_CODE_TEXT,CNS_ON_STUDY_INITIAL_DIAGNOSIS.SUPPTU_QVAL_TUPTDZSTG</t>
   </si>
   <si>
     <t>COG_UPR_DX.REG_STAGE_CODE_TEXT</t>
@@ -1629,7 +1626,7 @@
         <v>9</v>
       </c>
       <c r="K1" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
@@ -1643,7 +1640,7 @@
         <v>11</v>
       </c>
       <c r="E2" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F2" t="s">
         <v>26</v>
@@ -1732,16 +1729,16 @@
         <v>11</v>
       </c>
       <c r="E6" t="s">
+        <v>216</v>
+      </c>
+      <c r="F6" t="s">
+        <v>26</v>
+      </c>
+      <c r="H6" t="s">
+        <v>26</v>
+      </c>
+      <c r="I6" t="s">
         <v>217</v>
-      </c>
-      <c r="F6" t="s">
-        <v>26</v>
-      </c>
-      <c r="H6" t="s">
-        <v>26</v>
-      </c>
-      <c r="I6" t="s">
-        <v>218</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
@@ -1755,7 +1752,7 @@
         <v>20</v>
       </c>
       <c r="E7" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F7" t="s">
         <v>26</v>
@@ -1807,10 +1804,10 @@
         <v>22</v>
       </c>
       <c r="H9" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J9" t="s">
         <v>17</v>
@@ -1830,7 +1827,7 @@
         <v>23</v>
       </c>
       <c r="F10" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G10" t="s">
         <v>24</v>
@@ -1908,7 +1905,7 @@
         <v>17</v>
       </c>
       <c r="K13" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.2">
@@ -2091,7 +2088,7 @@
         <v>20</v>
       </c>
       <c r="E22" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F22" t="s">
         <v>26</v>
@@ -2149,10 +2146,10 @@
         <v>52</v>
       </c>
       <c r="H24" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="I24" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J24" t="s">
         <v>17</v>
@@ -2172,7 +2169,7 @@
         <v>23</v>
       </c>
       <c r="F25" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G25" t="s">
         <v>24</v>
@@ -2230,7 +2227,7 @@
         <v>17</v>
       </c>
       <c r="K27" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.2">
@@ -2319,7 +2316,7 @@
         <v>36</v>
       </c>
       <c r="G31" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.2">
@@ -2365,7 +2362,7 @@
         <v>42</v>
       </c>
       <c r="G33" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.2">
@@ -2445,7 +2442,7 @@
         <v>20</v>
       </c>
       <c r="E37" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F37" t="s">
         <v>26</v>
@@ -2500,10 +2497,10 @@
         <v>58</v>
       </c>
       <c r="H39" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="I39" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J39" t="s">
         <v>17</v>
@@ -2523,7 +2520,7 @@
         <v>23</v>
       </c>
       <c r="F40" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G40" t="s">
         <v>24</v>
@@ -2595,7 +2592,7 @@
         <v>31</v>
       </c>
       <c r="G43" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J43" t="s">
         <v>17</v>
@@ -2658,7 +2655,7 @@
         <v>36</v>
       </c>
       <c r="G46" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.2">
@@ -2750,7 +2747,7 @@
         <v>73</v>
       </c>
       <c r="I50" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.2">
@@ -2787,7 +2784,7 @@
         <v>20</v>
       </c>
       <c r="E52" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F52" t="s">
         <v>26</v>
@@ -2842,10 +2839,10 @@
         <v>52</v>
       </c>
       <c r="H54" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="I54" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J54" t="s">
         <v>17</v>
@@ -2865,10 +2862,10 @@
         <v>23</v>
       </c>
       <c r="F55" t="s">
+        <v>162</v>
+      </c>
+      <c r="G55" t="s">
         <v>163</v>
-      </c>
-      <c r="G55" t="s">
-        <v>164</v>
       </c>
       <c r="J55" t="s">
         <v>54</v>
@@ -2917,7 +2914,7 @@
         <v>36</v>
       </c>
       <c r="G57" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="J57" t="s">
         <v>17</v>
@@ -2940,7 +2937,7 @@
         <v>31</v>
       </c>
       <c r="G58" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.2">
@@ -2960,7 +2957,7 @@
         <v>36</v>
       </c>
       <c r="G59" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.2">
@@ -3138,7 +3135,7 @@
         <v>20</v>
       </c>
       <c r="E67" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F67" t="s">
         <v>26</v>
@@ -3193,10 +3190,10 @@
         <v>58</v>
       </c>
       <c r="H69" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="I69" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J69" t="s">
         <v>17</v>
@@ -3216,10 +3213,10 @@
         <v>23</v>
       </c>
       <c r="F70" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G70" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.2">
@@ -3288,7 +3285,7 @@
         <v>31</v>
       </c>
       <c r="G73" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="74" spans="1:10" x14ac:dyDescent="0.2">
@@ -3308,7 +3305,7 @@
         <v>36</v>
       </c>
       <c r="G74" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.2">
@@ -3486,7 +3483,7 @@
         <v>20</v>
       </c>
       <c r="E82" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F82" t="s">
         <v>26</v>
@@ -3541,10 +3538,10 @@
         <v>79</v>
       </c>
       <c r="H84" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="I84" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="J84" t="s">
         <v>17</v>
@@ -3564,10 +3561,10 @@
         <v>23</v>
       </c>
       <c r="F85" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G85" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="J85" t="s">
         <v>54</v>
@@ -3616,7 +3613,7 @@
         <v>36</v>
       </c>
       <c r="G87" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="J87" t="s">
         <v>17</v>
@@ -3639,7 +3636,7 @@
         <v>31</v>
       </c>
       <c r="G88" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="89" spans="1:10" x14ac:dyDescent="0.2">
@@ -3659,7 +3656,7 @@
         <v>36</v>
       </c>
       <c r="G89" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="90" spans="1:10" x14ac:dyDescent="0.2">
@@ -3837,7 +3834,7 @@
         <v>20</v>
       </c>
       <c r="E97" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F97" t="s">
         <v>26</v>
@@ -3892,10 +3889,10 @@
         <v>58</v>
       </c>
       <c r="H99" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="I99" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J99" t="s">
         <v>17</v>
@@ -3915,7 +3912,7 @@
         <v>23</v>
       </c>
       <c r="F100" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G100" t="s">
         <v>24</v>
@@ -3990,7 +3987,7 @@
         <v>26</v>
       </c>
       <c r="I103" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="104" spans="1:10" x14ac:dyDescent="0.2">
@@ -4059,7 +4056,7 @@
         <v>36</v>
       </c>
       <c r="G106" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="107" spans="1:10" x14ac:dyDescent="0.2">
@@ -4194,7 +4191,7 @@
         <v>20</v>
       </c>
       <c r="E112" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F112" t="s">
         <v>26</v>
@@ -4249,10 +4246,10 @@
         <v>52</v>
       </c>
       <c r="H114" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="I114" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J114" t="s">
         <v>17</v>
@@ -4272,7 +4269,7 @@
         <v>23</v>
       </c>
       <c r="F115" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G115" t="s">
         <v>24</v>
@@ -4350,7 +4347,7 @@
         <v>26</v>
       </c>
       <c r="I118" s="1" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="119" spans="1:10" x14ac:dyDescent="0.2">
@@ -4465,7 +4462,7 @@
         <v>42</v>
       </c>
       <c r="G123" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="124" spans="1:10" x14ac:dyDescent="0.2">
@@ -4545,7 +4542,7 @@
         <v>20</v>
       </c>
       <c r="E127" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F127" t="s">
         <v>26</v>
@@ -4600,10 +4597,10 @@
         <v>79</v>
       </c>
       <c r="H129" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="I129" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="J129" t="s">
         <v>17</v>
@@ -4623,7 +4620,7 @@
         <v>23</v>
       </c>
       <c r="F130" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G130" t="s">
         <v>24</v>
@@ -4698,7 +4695,7 @@
         <v>26</v>
       </c>
       <c r="I133" s="1" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="134" spans="1:10" x14ac:dyDescent="0.2">
@@ -4813,7 +4810,7 @@
         <v>42</v>
       </c>
       <c r="G138" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="139" spans="1:10" x14ac:dyDescent="0.2">
@@ -4899,7 +4896,7 @@
         <v>20</v>
       </c>
       <c r="E142" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F142" t="s">
         <v>26</v>
@@ -4957,10 +4954,10 @@
         <v>79</v>
       </c>
       <c r="H144" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="I144" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="J144" t="s">
         <v>17</v>
@@ -4980,7 +4977,7 @@
         <v>23</v>
       </c>
       <c r="F145" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G145" t="s">
         <v>24</v>
@@ -5055,7 +5052,7 @@
         <v>31</v>
       </c>
       <c r="G148" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J148" t="s">
         <v>17</v>
@@ -5250,13 +5247,13 @@
         <v>10</v>
       </c>
       <c r="B157" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D157" t="s">
         <v>20</v>
       </c>
       <c r="E157" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F157" t="s">
         <v>26</v>
@@ -5273,7 +5270,7 @@
         <v>10</v>
       </c>
       <c r="B158" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D158" t="s">
         <v>20</v>
@@ -5296,7 +5293,7 @@
         <v>10</v>
       </c>
       <c r="B159" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D159" t="s">
         <v>20</v>
@@ -5311,10 +5308,10 @@
         <v>22</v>
       </c>
       <c r="H159" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="I159" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J159" t="s">
         <v>17</v>
@@ -5325,7 +5322,7 @@
         <v>10</v>
       </c>
       <c r="B160" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D160" t="s">
         <v>20</v>
@@ -5334,10 +5331,10 @@
         <v>23</v>
       </c>
       <c r="F160" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G160" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="161" spans="1:10" x14ac:dyDescent="0.2">
@@ -5345,7 +5342,7 @@
         <v>10</v>
       </c>
       <c r="B161" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D161" t="s">
         <v>20</v>
@@ -5368,7 +5365,7 @@
         <v>10</v>
       </c>
       <c r="B162" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C162" t="b">
         <v>1</v>
@@ -5383,7 +5380,7 @@
         <v>36</v>
       </c>
       <c r="G162" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="J162" t="s">
         <v>17</v>
@@ -5394,7 +5391,7 @@
         <v>10</v>
       </c>
       <c r="B163" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D163" t="s">
         <v>20</v>
@@ -5406,7 +5403,7 @@
         <v>31</v>
       </c>
       <c r="G163" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="164" spans="1:10" x14ac:dyDescent="0.2">
@@ -5414,7 +5411,7 @@
         <v>10</v>
       </c>
       <c r="B164" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D164" t="s">
         <v>20</v>
@@ -5426,7 +5423,7 @@
         <v>36</v>
       </c>
       <c r="G164" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="165" spans="1:10" x14ac:dyDescent="0.2">
@@ -5434,7 +5431,7 @@
         <v>10</v>
       </c>
       <c r="B165" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D165" t="s">
         <v>20</v>
@@ -5457,7 +5454,7 @@
         <v>10</v>
       </c>
       <c r="B166" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D166" t="s">
         <v>20</v>
@@ -5480,7 +5477,7 @@
         <v>10</v>
       </c>
       <c r="B167" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D167" t="s">
         <v>20</v>
@@ -5503,7 +5500,7 @@
         <v>10</v>
       </c>
       <c r="B168" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D168" t="s">
         <v>20</v>
@@ -5526,7 +5523,7 @@
         <v>10</v>
       </c>
       <c r="B169" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D169" t="s">
         <v>20</v>
@@ -5549,7 +5546,7 @@
         <v>10</v>
       </c>
       <c r="B170" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D170" t="s">
         <v>20</v>
@@ -5575,7 +5572,7 @@
         <v>10</v>
       </c>
       <c r="B171" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D171" t="s">
         <v>20</v>
@@ -5598,13 +5595,13 @@
         <v>10</v>
       </c>
       <c r="B172" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D172" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E172" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F172" t="s">
         <v>26</v>
@@ -5613,7 +5610,7 @@
         <v>26</v>
       </c>
       <c r="I172" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="173" spans="1:10" x14ac:dyDescent="0.2">
@@ -5621,10 +5618,10 @@
         <v>10</v>
       </c>
       <c r="B173" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D173" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E173" s="2" t="s">
         <v>72</v>
@@ -5641,25 +5638,25 @@
         <v>10</v>
       </c>
       <c r="B174" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D174" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E174" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F174" t="s">
         <v>74</v>
       </c>
       <c r="G174" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H174" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="I174" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="175" spans="1:10" x14ac:dyDescent="0.2">
@@ -5667,22 +5664,22 @@
         <v>10</v>
       </c>
       <c r="B175" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C175" t="b">
         <v>1</v>
       </c>
       <c r="D175" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E175" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F175" t="s">
         <v>13</v>
       </c>
       <c r="G175" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="176" spans="1:10" x14ac:dyDescent="0.2">
@@ -5690,19 +5687,19 @@
         <v>10</v>
       </c>
       <c r="B176" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D176" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E176" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F176" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G176" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="177" spans="1:11" x14ac:dyDescent="0.2">
@@ -5710,22 +5707,22 @@
         <v>10</v>
       </c>
       <c r="B177" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D177" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E177" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F177" t="s">
         <v>36</v>
       </c>
       <c r="G177" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="K177" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="178" spans="1:11" x14ac:dyDescent="0.2">
@@ -5733,19 +5730,19 @@
         <v>10</v>
       </c>
       <c r="B178" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D178" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E178" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F178" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="G178" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="179" spans="1:11" x14ac:dyDescent="0.2">
@@ -5753,19 +5750,19 @@
         <v>10</v>
       </c>
       <c r="B179" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D179" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E179" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F179" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G179" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="180" spans="1:11" x14ac:dyDescent="0.2">
@@ -5773,13 +5770,13 @@
         <v>10</v>
       </c>
       <c r="B180" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D180" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E180" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F180" t="s">
         <v>26</v>
@@ -5793,13 +5790,13 @@
         <v>10</v>
       </c>
       <c r="B181" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D181" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E181" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F181" t="s">
         <v>26</v>
@@ -5813,13 +5810,13 @@
         <v>10</v>
       </c>
       <c r="B182" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D182" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E182" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F182" t="s">
         <v>26</v>
@@ -5833,13 +5830,13 @@
         <v>10</v>
       </c>
       <c r="B183" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D183" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E183" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F183" t="s">
         <v>26</v>
@@ -5853,13 +5850,13 @@
         <v>10</v>
       </c>
       <c r="B184" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D184" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E184" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F184" t="s">
         <v>26</v>
@@ -5873,13 +5870,13 @@
         <v>10</v>
       </c>
       <c r="B185" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D185" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E185" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="F185" t="s">
         <v>26</v>
@@ -5893,13 +5890,13 @@
         <v>10</v>
       </c>
       <c r="B186" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D186" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E186" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="F186" t="s">
         <v>26</v>
@@ -5913,13 +5910,13 @@
         <v>10</v>
       </c>
       <c r="B187" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D187" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E187" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F187" t="s">
         <v>26</v>
@@ -5928,7 +5925,7 @@
         <v>26</v>
       </c>
       <c r="I187" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="188" spans="1:11" x14ac:dyDescent="0.2">
@@ -5936,10 +5933,10 @@
         <v>10</v>
       </c>
       <c r="B188" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D188" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E188" s="2" t="s">
         <v>72</v>
@@ -5956,31 +5953,31 @@
         <v>10</v>
       </c>
       <c r="B189" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D189" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E189" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F189" t="s">
         <v>74</v>
       </c>
       <c r="G189" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H189" t="s">
+        <v>178</v>
+      </c>
+      <c r="I189" t="s">
         <v>179</v>
       </c>
-      <c r="I189" t="s">
-        <v>180</v>
-      </c>
       <c r="J189" t="s">
         <v>17</v>
       </c>
       <c r="K189" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="190" spans="1:11" x14ac:dyDescent="0.2">
@@ -5988,19 +5985,19 @@
         <v>10</v>
       </c>
       <c r="B190" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D190" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E190" s="2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F190" t="s">
+        <v>182</v>
+      </c>
+      <c r="G190" t="s">
         <v>183</v>
-      </c>
-      <c r="G190" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="191" spans="1:11" x14ac:dyDescent="0.2">
@@ -6008,13 +6005,13 @@
         <v>10</v>
       </c>
       <c r="B191" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D191" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E191" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F191" t="s">
         <v>26</v>
@@ -6031,13 +6028,13 @@
         <v>10</v>
       </c>
       <c r="B192" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D192" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E192" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F192" t="s">
         <v>26</v>
@@ -6054,13 +6051,13 @@
         <v>10</v>
       </c>
       <c r="B193" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D193" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E193" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="F193" t="s">
         <v>26</v>
@@ -6077,13 +6074,13 @@
         <v>10</v>
       </c>
       <c r="B194" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D194" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E194" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F194" t="s">
         <v>26</v>
@@ -6092,7 +6089,7 @@
         <v>26</v>
       </c>
       <c r="I194" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="195" spans="1:10" x14ac:dyDescent="0.2">
@@ -6100,10 +6097,10 @@
         <v>10</v>
       </c>
       <c r="B195" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D195" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E195" s="2" t="s">
         <v>72</v>
@@ -6120,13 +6117,13 @@
         <v>10</v>
       </c>
       <c r="B196" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D196" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E196" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F196" t="s">
         <v>13</v>
@@ -6138,7 +6135,7 @@
         <v>73</v>
       </c>
       <c r="I196" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="197" spans="1:10" x14ac:dyDescent="0.2">
@@ -6146,13 +6143,13 @@
         <v>10</v>
       </c>
       <c r="B197" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D197" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E197" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F197" t="s">
         <v>26</v>
@@ -6161,7 +6158,7 @@
         <v>26</v>
       </c>
       <c r="I197" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="198" spans="1:10" x14ac:dyDescent="0.2">
@@ -6169,28 +6166,28 @@
         <v>10</v>
       </c>
       <c r="B198" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C198" t="b">
         <v>1</v>
       </c>
       <c r="D198" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E198" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F198" t="s">
         <v>36</v>
       </c>
       <c r="G198" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="H198" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="I198" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="199" spans="1:10" x14ac:dyDescent="0.2">
@@ -6198,13 +6195,13 @@
         <v>10</v>
       </c>
       <c r="B199" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D199" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E199" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F199" t="s">
         <v>26</v>
@@ -6221,13 +6218,13 @@
         <v>10</v>
       </c>
       <c r="B200" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D200" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E200" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F200" t="s">
         <v>26</v>
@@ -6247,19 +6244,19 @@
         <v>10</v>
       </c>
       <c r="B201" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D201" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E201" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F201" t="s">
         <v>36</v>
       </c>
       <c r="G201" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="202" spans="1:10" x14ac:dyDescent="0.2">
@@ -6267,13 +6264,13 @@
         <v>10</v>
       </c>
       <c r="B202" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D202" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E202" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F202" t="s">
         <v>26</v>
@@ -6287,13 +6284,13 @@
         <v>10</v>
       </c>
       <c r="B203" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D203" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E203" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F203" t="s">
         <v>26</v>
@@ -6307,10 +6304,10 @@
         <v>10</v>
       </c>
       <c r="B204" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D204" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E204" s="3" t="s">
         <v>33</v>
@@ -6330,10 +6327,10 @@
         <v>10</v>
       </c>
       <c r="B205" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D205" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E205" s="3" t="s">
         <v>33</v>
@@ -6350,13 +6347,13 @@
         <v>10</v>
       </c>
       <c r="B206" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D206" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E206" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F206" t="s">
         <v>26</v>
@@ -6365,7 +6362,7 @@
         <v>26</v>
       </c>
       <c r="I206" s="4" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="207" spans="1:10" x14ac:dyDescent="0.2">
@@ -6373,13 +6370,13 @@
         <v>10</v>
       </c>
       <c r="B207" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D207" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E207" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F207" t="s">
         <v>26</v>
@@ -6393,13 +6390,13 @@
         <v>10</v>
       </c>
       <c r="B208" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D208" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E208" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F208" t="s">
         <v>26</v>
@@ -6413,13 +6410,13 @@
         <v>10</v>
       </c>
       <c r="B209" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D209" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E209" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F209" t="s">
         <v>26</v>
@@ -6433,13 +6430,13 @@
         <v>10</v>
       </c>
       <c r="B210" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D210" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E210" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F210" t="s">
         <v>26</v>
@@ -6448,7 +6445,7 @@
         <v>26</v>
       </c>
       <c r="I210" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="211" spans="1:10" x14ac:dyDescent="0.2">
@@ -6456,10 +6453,10 @@
         <v>10</v>
       </c>
       <c r="B211" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D211" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E211" s="2" t="s">
         <v>72</v>
@@ -6476,13 +6473,13 @@
         <v>10</v>
       </c>
       <c r="B212" t="s">
+        <v>117</v>
+      </c>
+      <c r="D212" t="s">
+        <v>117</v>
+      </c>
+      <c r="E212" s="2" t="s">
         <v>118</v>
-      </c>
-      <c r="D212" t="s">
-        <v>118</v>
-      </c>
-      <c r="E212" s="2" t="s">
-        <v>119</v>
       </c>
       <c r="F212" t="s">
         <v>13</v>
@@ -6494,7 +6491,7 @@
         <v>73</v>
       </c>
       <c r="I212" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="213" spans="1:10" x14ac:dyDescent="0.2">
@@ -6502,13 +6499,13 @@
         <v>10</v>
       </c>
       <c r="B213" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D213" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E213" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F213" t="s">
         <v>26</v>
@@ -6525,22 +6522,22 @@
         <v>10</v>
       </c>
       <c r="B214" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C214" t="b">
         <v>1</v>
       </c>
       <c r="D214" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E214" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F214" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G214" s="2" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="215" spans="1:10" x14ac:dyDescent="0.2">
@@ -6548,13 +6545,13 @@
         <v>10</v>
       </c>
       <c r="B215" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D215" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E215" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F215" t="s">
         <v>26</v>
@@ -6571,13 +6568,13 @@
         <v>10</v>
       </c>
       <c r="B216" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D216" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E216" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F216" t="s">
         <v>26</v>
@@ -6594,13 +6591,13 @@
         <v>10</v>
       </c>
       <c r="B217" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D217" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E217" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F217" t="s">
         <v>26</v>
@@ -6609,7 +6606,7 @@
         <v>26</v>
       </c>
       <c r="I217" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="218" spans="1:10" x14ac:dyDescent="0.2">
@@ -6617,10 +6614,10 @@
         <v>10</v>
       </c>
       <c r="B218" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D218" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E218" s="2" t="s">
         <v>72</v>
@@ -6637,13 +6634,13 @@
         <v>10</v>
       </c>
       <c r="B219" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D219" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E219" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F219" t="s">
         <v>13</v>
@@ -6655,7 +6652,7 @@
         <v>73</v>
       </c>
       <c r="I219" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="220" spans="1:10" x14ac:dyDescent="0.2">
@@ -6663,13 +6660,13 @@
         <v>10</v>
       </c>
       <c r="B220" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D220" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E220" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F220" t="s">
         <v>26</v>
@@ -6678,10 +6675,10 @@
         <v>26</v>
       </c>
       <c r="I220" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="J220" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="221" spans="1:10" x14ac:dyDescent="0.2">
@@ -6689,25 +6686,25 @@
         <v>10</v>
       </c>
       <c r="B221" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C221" t="b">
         <v>1</v>
       </c>
       <c r="D221" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E221" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F221" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G221" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="J221" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="222" spans="1:10" x14ac:dyDescent="0.2">
@@ -6715,19 +6712,19 @@
         <v>10</v>
       </c>
       <c r="B222" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D222" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E222" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F222" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G222" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="J222">
         <v>-999</v>
@@ -6738,19 +6735,19 @@
         <v>10</v>
       </c>
       <c r="B223" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D223" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E223" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F223" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G223" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="J223">
         <v>-999</v>
@@ -6761,13 +6758,13 @@
         <v>10</v>
       </c>
       <c r="B224" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D224" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E224" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F224" t="s">
         <v>26</v>
@@ -6784,22 +6781,22 @@
         <v>10</v>
       </c>
       <c r="B225" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D225" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E225" s="3" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F225" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G225" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="I225" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="226" spans="1:9" x14ac:dyDescent="0.2">
@@ -6807,13 +6804,13 @@
         <v>10</v>
       </c>
       <c r="B226" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D226" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E226" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F226" t="s">
         <v>26</v>
@@ -6822,7 +6819,7 @@
         <v>26</v>
       </c>
       <c r="I226" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="227" spans="1:9" x14ac:dyDescent="0.2">
@@ -6830,10 +6827,10 @@
         <v>10</v>
       </c>
       <c r="B227" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D227" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E227" s="3" t="s">
         <v>72</v>
@@ -6850,13 +6847,13 @@
         <v>10</v>
       </c>
       <c r="B228" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D228" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E228" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F228" t="s">
         <v>13</v>
@@ -6868,7 +6865,7 @@
         <v>73</v>
       </c>
       <c r="I228" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="229" spans="1:9" x14ac:dyDescent="0.2">
@@ -6876,13 +6873,13 @@
         <v>10</v>
       </c>
       <c r="B229" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D229" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E229" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F229" t="s">
         <v>26</v>
@@ -6891,7 +6888,7 @@
         <v>26</v>
       </c>
       <c r="I229" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="230" spans="1:9" x14ac:dyDescent="0.2">
@@ -6899,22 +6896,22 @@
         <v>10</v>
       </c>
       <c r="B230" t="s">
+        <v>194</v>
+      </c>
+      <c r="D230" t="s">
+        <v>105</v>
+      </c>
+      <c r="E230" s="3" t="s">
+        <v>214</v>
+      </c>
+      <c r="F230" t="s">
+        <v>26</v>
+      </c>
+      <c r="H230" t="s">
+        <v>26</v>
+      </c>
+      <c r="I230" t="s">
         <v>195</v>
-      </c>
-      <c r="D230" t="s">
-        <v>106</v>
-      </c>
-      <c r="E230" s="3" t="s">
-        <v>215</v>
-      </c>
-      <c r="F230" t="s">
-        <v>26</v>
-      </c>
-      <c r="H230" t="s">
-        <v>26</v>
-      </c>
-      <c r="I230" t="s">
-        <v>196</v>
       </c>
     </row>
     <row r="231" spans="1:9" x14ac:dyDescent="0.2">
@@ -6922,13 +6919,13 @@
         <v>10</v>
       </c>
       <c r="B231" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D231" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E231" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F231" t="s">
         <v>26</v>
@@ -6945,13 +6942,13 @@
         <v>10</v>
       </c>
       <c r="B232" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D232" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E232" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F232" t="s">
         <v>26</v>
@@ -6968,22 +6965,22 @@
         <v>10</v>
       </c>
       <c r="B233" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C233" t="b">
         <v>1</v>
       </c>
       <c r="D233" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E233" s="3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F233" t="s">
         <v>36</v>
       </c>
       <c r="G233" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="234" spans="1:9" x14ac:dyDescent="0.2">
@@ -6991,13 +6988,13 @@
         <v>10</v>
       </c>
       <c r="B234" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D234" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E234" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F234" t="s">
         <v>26</v>
@@ -7011,13 +7008,13 @@
         <v>10</v>
       </c>
       <c r="B235" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D235" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E235" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F235" t="s">
         <v>26</v>
@@ -7031,13 +7028,13 @@
         <v>10</v>
       </c>
       <c r="B236" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D236" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E236" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F236" t="s">
         <v>26</v>
@@ -7051,13 +7048,13 @@
         <v>10</v>
       </c>
       <c r="B237" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D237" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E237" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F237" t="s">
         <v>26</v>
@@ -7071,13 +7068,13 @@
         <v>10</v>
       </c>
       <c r="B238" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D238" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E238" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F238" t="s">
         <v>26</v>
@@ -7091,13 +7088,13 @@
         <v>10</v>
       </c>
       <c r="B239" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D239" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E239" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F239" t="s">
         <v>26</v>
@@ -7111,13 +7108,13 @@
         <v>10</v>
       </c>
       <c r="B240" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D240" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E240" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F240" t="s">
         <v>26</v>
@@ -7131,13 +7128,13 @@
         <v>10</v>
       </c>
       <c r="B241" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D241" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E241" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F241" t="s">
         <v>26</v>
@@ -7146,7 +7143,7 @@
         <v>26</v>
       </c>
       <c r="I241" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="242" spans="1:9" x14ac:dyDescent="0.2">
@@ -7154,10 +7151,10 @@
         <v>10</v>
       </c>
       <c r="B242" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D242" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E242" s="2" t="s">
         <v>72</v>
@@ -7174,13 +7171,13 @@
         <v>10</v>
       </c>
       <c r="B243" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D243" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E243" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F243" t="s">
         <v>13</v>
@@ -7192,7 +7189,7 @@
         <v>73</v>
       </c>
       <c r="I243" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="244" spans="1:9" x14ac:dyDescent="0.2">
@@ -7200,13 +7197,13 @@
         <v>10</v>
       </c>
       <c r="B244" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D244" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E244" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F244" t="s">
         <v>26</v>
@@ -7215,7 +7212,7 @@
         <v>26</v>
       </c>
       <c r="I244" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="245" spans="1:9" x14ac:dyDescent="0.2">
@@ -7223,13 +7220,13 @@
         <v>10</v>
       </c>
       <c r="B245" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D245" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E245" s="2" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="F245" t="s">
         <v>26</v>
@@ -7238,7 +7235,7 @@
         <v>26</v>
       </c>
       <c r="I245" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="246" spans="1:9" x14ac:dyDescent="0.2">
@@ -7246,13 +7243,13 @@
         <v>10</v>
       </c>
       <c r="B246" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D246" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E246" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F246" t="s">
         <v>26</v>
@@ -7269,13 +7266,13 @@
         <v>10</v>
       </c>
       <c r="B247" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D247" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E247" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F247" t="s">
         <v>26</v>
@@ -7292,22 +7289,22 @@
         <v>10</v>
       </c>
       <c r="B248" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C248" t="b">
         <v>1</v>
       </c>
       <c r="D248" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E248" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F248" t="s">
         <v>36</v>
       </c>
       <c r="G248" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="249" spans="1:9" x14ac:dyDescent="0.2">
@@ -7315,13 +7312,13 @@
         <v>10</v>
       </c>
       <c r="B249" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D249" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E249" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F249" t="s">
         <v>26</v>
@@ -7335,13 +7332,13 @@
         <v>10</v>
       </c>
       <c r="B250" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D250" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E250" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F250" t="s">
         <v>26</v>
@@ -7355,13 +7352,13 @@
         <v>10</v>
       </c>
       <c r="B251" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D251" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E251" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F251" t="s">
         <v>26</v>
@@ -7375,13 +7372,13 @@
         <v>10</v>
       </c>
       <c r="B252" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D252" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E252" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F252" t="s">
         <v>26</v>
@@ -7395,13 +7392,13 @@
         <v>10</v>
       </c>
       <c r="B253" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D253" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E253" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F253" t="s">
         <v>26</v>
@@ -7415,13 +7412,13 @@
         <v>10</v>
       </c>
       <c r="B254" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D254" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E254" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F254" t="s">
         <v>26</v>
@@ -7435,13 +7432,13 @@
         <v>10</v>
       </c>
       <c r="B255" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D255" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E255" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F255" t="s">
         <v>26</v>
@@ -7455,13 +7452,13 @@
         <v>10</v>
       </c>
       <c r="B256" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D256" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E256" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F256" t="s">
         <v>26</v>
@@ -7470,7 +7467,7 @@
         <v>26</v>
       </c>
       <c r="I256" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="257" spans="1:9" x14ac:dyDescent="0.2">
@@ -7478,10 +7475,10 @@
         <v>10</v>
       </c>
       <c r="B257" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D257" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E257" s="2" t="s">
         <v>72</v>
@@ -7498,13 +7495,13 @@
         <v>10</v>
       </c>
       <c r="B258" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D258" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E258" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F258" t="s">
         <v>13</v>
@@ -7516,7 +7513,7 @@
         <v>73</v>
       </c>
       <c r="I258" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="259" spans="1:9" x14ac:dyDescent="0.2">
@@ -7524,13 +7521,13 @@
         <v>10</v>
       </c>
       <c r="B259" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D259" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E259" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F259" t="s">
         <v>26</v>
@@ -7539,7 +7536,7 @@
         <v>26</v>
       </c>
       <c r="I259" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="260" spans="1:9" x14ac:dyDescent="0.2">
@@ -7547,13 +7544,13 @@
         <v>10</v>
       </c>
       <c r="B260" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D260" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E260" s="2" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="F260" t="s">
         <v>26</v>
@@ -7562,7 +7559,7 @@
         <v>26</v>
       </c>
       <c r="I260" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="261" spans="1:9" x14ac:dyDescent="0.2">
@@ -7570,13 +7567,13 @@
         <v>10</v>
       </c>
       <c r="B261" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D261" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E261" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F261" t="s">
         <v>26</v>
@@ -7593,13 +7590,13 @@
         <v>10</v>
       </c>
       <c r="B262" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D262" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E262" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F262" t="s">
         <v>26</v>
@@ -7616,22 +7613,22 @@
         <v>10</v>
       </c>
       <c r="B263" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C263" t="b">
         <v>1</v>
       </c>
       <c r="D263" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E263" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F263" t="s">
         <v>36</v>
       </c>
       <c r="G263" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="264" spans="1:9" x14ac:dyDescent="0.2">
@@ -7639,13 +7636,13 @@
         <v>10</v>
       </c>
       <c r="B264" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D264" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E264" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F264" t="s">
         <v>26</v>
@@ -7659,13 +7656,13 @@
         <v>10</v>
       </c>
       <c r="B265" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D265" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E265" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F265" t="s">
         <v>26</v>
@@ -7679,13 +7676,13 @@
         <v>10</v>
       </c>
       <c r="B266" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D266" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E266" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F266" t="s">
         <v>26</v>
@@ -7699,13 +7696,13 @@
         <v>10</v>
       </c>
       <c r="B267" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D267" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E267" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F267" t="s">
         <v>26</v>
@@ -7719,13 +7716,13 @@
         <v>10</v>
       </c>
       <c r="B268" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D268" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E268" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F268" t="s">
         <v>26</v>
@@ -7739,13 +7736,13 @@
         <v>10</v>
       </c>
       <c r="B269" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D269" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E269" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F269" t="s">
         <v>26</v>
@@ -7759,13 +7756,13 @@
         <v>10</v>
       </c>
       <c r="B270" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D270" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E270" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F270" t="s">
         <v>26</v>
@@ -7779,13 +7776,13 @@
         <v>10</v>
       </c>
       <c r="B271" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D271" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E271" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F271" t="s">
         <v>26</v>
@@ -7794,7 +7791,7 @@
         <v>26</v>
       </c>
       <c r="I271" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="272" spans="1:9" x14ac:dyDescent="0.2">
@@ -7802,10 +7799,10 @@
         <v>10</v>
       </c>
       <c r="B272" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D272" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E272" s="2" t="s">
         <v>72</v>
@@ -7822,13 +7819,13 @@
         <v>10</v>
       </c>
       <c r="B273" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D273" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E273" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F273" t="s">
         <v>13</v>
@@ -7840,7 +7837,7 @@
         <v>73</v>
       </c>
       <c r="I273" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="274" spans="1:9" x14ac:dyDescent="0.2">
@@ -7848,13 +7845,13 @@
         <v>10</v>
       </c>
       <c r="B274" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D274" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E274" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F274" t="s">
         <v>26</v>
@@ -7863,7 +7860,7 @@
         <v>26</v>
       </c>
       <c r="I274" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="275" spans="1:9" x14ac:dyDescent="0.2">
@@ -7871,13 +7868,13 @@
         <v>10</v>
       </c>
       <c r="B275" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D275" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E275" s="2" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="F275" t="s">
         <v>26</v>
@@ -7886,7 +7883,7 @@
         <v>26</v>
       </c>
       <c r="I275" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="276" spans="1:9" x14ac:dyDescent="0.2">
@@ -7894,13 +7891,13 @@
         <v>10</v>
       </c>
       <c r="B276" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D276" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E276" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F276" t="s">
         <v>26</v>
@@ -7917,13 +7914,13 @@
         <v>10</v>
       </c>
       <c r="B277" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D277" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E277" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F277" t="s">
         <v>26</v>
@@ -7940,22 +7937,22 @@
         <v>10</v>
       </c>
       <c r="B278" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C278" t="b">
         <v>1</v>
       </c>
       <c r="D278" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E278" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F278" t="s">
         <v>36</v>
       </c>
       <c r="G278" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="279" spans="1:9" x14ac:dyDescent="0.2">
@@ -7963,13 +7960,13 @@
         <v>10</v>
       </c>
       <c r="B279" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D279" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E279" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F279" t="s">
         <v>26</v>
@@ -7983,13 +7980,13 @@
         <v>10</v>
       </c>
       <c r="B280" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D280" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E280" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F280" t="s">
         <v>26</v>
@@ -8003,13 +8000,13 @@
         <v>10</v>
       </c>
       <c r="B281" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D281" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E281" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F281" t="s">
         <v>26</v>
@@ -8023,13 +8020,13 @@
         <v>10</v>
       </c>
       <c r="B282" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D282" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E282" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F282" t="s">
         <v>26</v>
@@ -8043,13 +8040,13 @@
         <v>10</v>
       </c>
       <c r="B283" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D283" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E283" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F283" t="s">
         <v>26</v>
@@ -8063,13 +8060,13 @@
         <v>10</v>
       </c>
       <c r="B284" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D284" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E284" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F284" t="s">
         <v>26</v>
@@ -8083,13 +8080,13 @@
         <v>10</v>
       </c>
       <c r="B285" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D285" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E285" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F285" t="s">
         <v>26</v>
@@ -8103,13 +8100,13 @@
         <v>10</v>
       </c>
       <c r="B286" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D286" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E286" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F286" t="s">
         <v>26</v>
@@ -8118,7 +8115,7 @@
         <v>26</v>
       </c>
       <c r="I286" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="287" spans="1:9" x14ac:dyDescent="0.2">
@@ -8126,10 +8123,10 @@
         <v>10</v>
       </c>
       <c r="B287" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D287" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E287" s="2" t="s">
         <v>72</v>
@@ -8146,19 +8143,19 @@
         <v>10</v>
       </c>
       <c r="B288" t="s">
+        <v>209</v>
+      </c>
+      <c r="D288" t="s">
+        <v>105</v>
+      </c>
+      <c r="E288" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="F288" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="G288" s="2" t="s">
         <v>210</v>
-      </c>
-      <c r="D288" t="s">
-        <v>106</v>
-      </c>
-      <c r="E288" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="F288" s="2" t="s">
-        <v>213</v>
-      </c>
-      <c r="G288" s="2" t="s">
-        <v>211</v>
       </c>
       <c r="H288" s="2"/>
       <c r="I288" s="2"/>
@@ -8168,13 +8165,13 @@
         <v>10</v>
       </c>
       <c r="B289" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D289" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E289" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F289" s="2" t="s">
         <v>26</v>
@@ -8183,7 +8180,7 @@
         <v>26</v>
       </c>
       <c r="I289" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="290" spans="1:9" x14ac:dyDescent="0.2">
@@ -8191,19 +8188,19 @@
         <v>10</v>
       </c>
       <c r="B290" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D290" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E290" s="2" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="F290" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="G290" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="291" spans="1:9" x14ac:dyDescent="0.2">
@@ -8211,13 +8208,13 @@
         <v>10</v>
       </c>
       <c r="B291" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D291" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E291" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F291" t="s">
         <v>26</v>
@@ -8234,13 +8231,13 @@
         <v>10</v>
       </c>
       <c r="B292" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D292" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E292" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F292" t="s">
         <v>26</v>
@@ -8257,22 +8254,22 @@
         <v>10</v>
       </c>
       <c r="B293" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C293" t="b">
         <v>1</v>
       </c>
       <c r="D293" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E293" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F293" s="2" t="s">
         <v>13</v>
       </c>
       <c r="G293" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="294" spans="1:9" x14ac:dyDescent="0.2">
@@ -8280,13 +8277,13 @@
         <v>10</v>
       </c>
       <c r="B294" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D294" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E294" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F294" t="s">
         <v>26</v>
@@ -8300,13 +8297,13 @@
         <v>10</v>
       </c>
       <c r="B295" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D295" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E295" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F295" t="s">
         <v>26</v>
@@ -8320,13 +8317,13 @@
         <v>10</v>
       </c>
       <c r="B296" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D296" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E296" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F296" t="s">
         <v>26</v>
@@ -8340,13 +8337,13 @@
         <v>10</v>
       </c>
       <c r="B297" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D297" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E297" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F297" t="s">
         <v>26</v>
@@ -8360,13 +8357,13 @@
         <v>10</v>
       </c>
       <c r="B298" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D298" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E298" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F298" t="s">
         <v>26</v>
@@ -8380,13 +8377,13 @@
         <v>10</v>
       </c>
       <c r="B299" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D299" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E299" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F299" t="s">
         <v>26</v>
@@ -8400,13 +8397,13 @@
         <v>10</v>
       </c>
       <c r="B300" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D300" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E300" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F300" t="s">
         <v>26</v>
@@ -8435,7 +8432,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -8443,7 +8440,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
@@ -8451,7 +8448,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
@@ -8459,7 +8456,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
@@ -8467,7 +8464,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
@@ -8475,7 +8472,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
@@ -8483,7 +8480,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
@@ -8491,7 +8488,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
@@ -8499,7 +8496,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
@@ -8507,7 +8504,7 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
   </sheetData>

</xml_diff>